<commit_message>
added single and triple ship results, need to update numpy seed each ship run
</commit_message>
<xml_diff>
--- a/researchQuestions/simple_test_ship_data.xlsx
+++ b/researchQuestions/simple_test_ship_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adware\Desktop\KISS\researchQuestions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F2FFDA7-40A7-482C-B233-5525D2EB2DD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6DB838-85EA-4570-9004-27CDB67F6AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="735" windowWidth="14400" windowHeight="8183" xr2:uid="{279480E9-DBDF-4252-B432-4CE1D30BF378}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{279480E9-DBDF-4252-B432-4CE1D30BF378}"/>
   </bookViews>
   <sheets>
     <sheet name="machinery reliability data" sheetId="1" r:id="rId1"/>
@@ -540,16 +540,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F997A0B-9C86-4EC5-9A0F-10545207BFB0}">
   <dimension ref="A1:F37"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.73046875" customWidth="1"/>
-    <col min="2" max="2" width="24.1328125" customWidth="1"/>
-    <col min="3" max="3" width="18.265625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="18.86328125" customWidth="1"/>
-    <col min="5" max="6" width="18.265625" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" customWidth="1"/>
+    <col min="5" max="6" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
@@ -565,7 +565,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -573,13 +573,13 @@
         <v>8</v>
       </c>
       <c r="C2" s="2">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D2">
         <v>2.5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -587,13 +587,13 @@
         <v>9</v>
       </c>
       <c r="C3" s="2">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D3">
         <v>2.5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -601,13 +601,13 @@
         <v>10</v>
       </c>
       <c r="C4" s="2">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D4">
         <v>2.5</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -615,13 +615,13 @@
         <v>11</v>
       </c>
       <c r="C5" s="2">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D5">
         <v>2.5</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -629,13 +629,13 @@
         <v>12</v>
       </c>
       <c r="C6" s="2">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D6">
         <v>2.5</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -643,13 +643,13 @@
         <v>13</v>
       </c>
       <c r="C7" s="2">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D7">
         <v>2.5</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -657,13 +657,13 @@
         <v>14</v>
       </c>
       <c r="C8" s="2">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D8">
         <v>2.5</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -671,13 +671,13 @@
         <v>15</v>
       </c>
       <c r="C9" s="2">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D9">
         <v>2.5</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -685,13 +685,13 @@
         <v>16</v>
       </c>
       <c r="C10" s="2">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D10">
         <v>2.5</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -699,13 +699,13 @@
         <v>17</v>
       </c>
       <c r="C11" s="2">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D11">
         <v>2.5</v>
       </c>
     </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.45">
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C37" s="5"/>
     </row>
   </sheetData>
@@ -718,12 +718,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD4FF0A7-4C32-4212-8D10-DADC32F7B7B8}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="32.3984375" customWidth="1"/>
+    <col min="2" max="3" width="32.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -734,7 +734,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -745,7 +745,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -756,7 +756,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D6" s="4"/>
     </row>
   </sheetData>
@@ -768,19 +768,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B338D18E-1C2C-4003-BC79-5462DE0704E2}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.1328125" customWidth="1"/>
-    <col min="2" max="2" width="30.3984375" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -793,14 +793,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A16644A-918D-4FF5-9CE2-44B4969116F9}">
   <dimension ref="B1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="22.1328125" customWidth="1"/>
-    <col min="3" max="3" width="20.1328125" customWidth="1"/>
+    <col min="2" max="2" width="22.140625" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B1">
         <v>2</v>
       </c>
@@ -811,7 +811,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2">
         <v>3</v>
       </c>
@@ -822,7 +822,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
added good vs bad sensor test for comps, system and ship; need to update sensedSystem simulate func for seriesComps
</commit_message>
<xml_diff>
--- a/researchQuestions/simple_test_ship_data.xlsx
+++ b/researchQuestions/simple_test_ship_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adware\Desktop\KISS\researchQuestions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6DB838-85EA-4570-9004-27CDB67F6AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD7BF401-D346-49D0-84A9-9374D9378BD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{279480E9-DBDF-4252-B432-4CE1D30BF378}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11160" activeTab="1" xr2:uid="{279480E9-DBDF-4252-B432-4CE1D30BF378}"/>
   </bookViews>
   <sheets>
     <sheet name="machinery reliability data" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Component</t>
   </si>
@@ -83,21 +83,6 @@
     <t>Comp 6</t>
   </si>
   <si>
-    <t>Comp 7</t>
-  </si>
-  <si>
-    <t>Comp 8</t>
-  </si>
-  <si>
-    <t>Comp 9</t>
-  </si>
-  <si>
-    <t>Comp 10</t>
-  </si>
-  <si>
-    <t>[1,2,3,4]</t>
-  </si>
-  <si>
     <t>series - parallel system #1</t>
   </si>
   <si>
@@ -107,15 +92,6 @@
     <t>[(1,2,3,4)]</t>
   </si>
   <si>
-    <t>series system #2</t>
-  </si>
-  <si>
-    <t>series system #1</t>
-  </si>
-  <si>
-    <t>[5,6,7,8]</t>
-  </si>
-  <si>
     <t>parallel system #1</t>
   </si>
   <si>
@@ -125,7 +101,22 @@
     <t>[([1,2,3], [4,5,6]), ([7,8], [7,8], 9,10]</t>
   </si>
   <si>
-    <t>[(0,1)]</t>
+    <t>sys #1</t>
+  </si>
+  <si>
+    <t>sys #2</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>&lt;-- no parallel systems</t>
+  </si>
+  <si>
+    <t>[0,1,2]</t>
+  </si>
+  <si>
+    <t>[3,4,5]</t>
   </si>
 </sst>
 </file>
@@ -573,10 +564,10 @@
         <v>8</v>
       </c>
       <c r="C2" s="2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D2">
-        <v>2.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -587,10 +578,10 @@
         <v>9</v>
       </c>
       <c r="C3" s="2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>2.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -601,10 +592,10 @@
         <v>10</v>
       </c>
       <c r="C4" s="2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D4">
-        <v>2.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -615,10 +606,10 @@
         <v>11</v>
       </c>
       <c r="C5" s="2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D5">
-        <v>2.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -629,10 +620,10 @@
         <v>12</v>
       </c>
       <c r="C6" s="2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D6">
-        <v>2.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -643,66 +634,10 @@
         <v>13</v>
       </c>
       <c r="C7" s="2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D7">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="2">
-        <v>10</v>
-      </c>
-      <c r="D8">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="2">
-        <v>10</v>
-      </c>
-      <c r="D9">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="2">
-        <v>10</v>
-      </c>
-      <c r="D10">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="2">
-        <v>10</v>
-      </c>
-      <c r="D11">
-        <v>2.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="3:3" x14ac:dyDescent="0.25">
@@ -739,10 +674,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -750,10 +685,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -782,7 +717,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -805,10 +743,10 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
@@ -816,10 +754,10 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
@@ -827,10 +765,10 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>